<commit_message>
Docs(excel): preuves site interne, DNS et commandes de démo
Met à jour la grille d'évaluation (OK VPN, bastion, DNS, site interne LAN)
avec explications, preuves terminal et scénario de soutenance.
</commit_message>
<xml_diff>
--- a/docs/criteres_evaluation_infrastructure.xlsx
+++ b/docs/criteres_evaluation_infrastructure.xlsx
@@ -719,12 +719,23 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Validation en attente: démontrer que le site interne n'est accessible qu'en LAN/VPN et refusé depuis Internet.</t>
+          <t>EXPLICATION: Site web interne (nginx sur bastion 192.168.10.11, LAN 192.168.10.0/24). Accessible uniquement depuis réseau interne/VPN, non exposé sur Internet.
+PREUVE COMPLÈTE (2026-05-28):
+- Avec accès interne (bastion/VPN): curl -I http://192.168.10.11 -&gt; HTTP/1.1 200 OK
+- Sans VPN depuis Mac: curl http://78.202.114.212:80 -&gt; timeout (non exposé)
+- Sans VPN depuis Mac: curl http://192.168.10.11:80 -&gt; timeout (IP privée inaccessible)
+COMMANDES DÉMO (soutenance):
+1) Connecter VPN + ssh bastion@192.168.102.103
+2) curl -I http://192.168.10.11   # doit répondre 200
+3) Déconnecter VPN
+4) curl -I --connect-timeout 5 http://78.202.114.212   # doit échouer
+5) curl -I --connect-timeout 5 http://192.168.10.11   # doit échouer
+6) Reconnecter VPN et refaire étape 2</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -734,7 +745,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs(excel): validation accès SSH public port 2222
Mise à jour des critères spécification_réseau2 et pare-feu réseau avec preuves nc/ssh et commandes de démo.
</commit_message>
<xml_diff>
--- a/docs/criteres_evaluation_infrastructure.xlsx
+++ b/docs/criteres_evaluation_infrastructure.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20360" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="20" yWindow="660" windowWidth="34560" windowHeight="20360" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Critères Évaluation" sheetId="1" state="visible" r:id="rId1"/>
@@ -58,9 +58,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,15 +440,15 @@
   <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="100" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" style="2" min="1" max="1"/>
+    <col width="120" customWidth="1" style="2" min="2" max="2"/>
+    <col width="12" customWidth="1" style="2" min="3" max="3"/>
+    <col width="100" customWidth="1" style="4" min="4" max="4"/>
+    <col width="15" customWidth="1" style="2" min="5" max="5"/>
+    <col width="12" customWidth="1" style="2" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="16" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Rubrique</t>
@@ -453,7 +464,7 @@
           <t>Statut</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Commentaires</t>
         </is>
@@ -469,55 +480,55 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>livraison_infrastructure</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Une infrastructure de cloud hybride est livrée ET fonctionnelle.</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>EXPLICATION: Infrastructure hybride = 2 sites Proxmox interconnectés VPN, sécurisés, observables. Partiellement fonctionnelle (VPN+bastion+DNS OK sur site distant). Manque site A complet, services transverses (NetBox/Elastic), démo bout-en-bout documentée.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="240" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>infra_spec</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>La grande majorité des services requis sont présents et fonctionnels.</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>EXPLICATION: Services requis du sujet CIA: 2 sites Proxmox, VPN, 2x pfSense, bastion, DNS, IPAM NetBox, Elastic, site web interne.
 DÉJÀ EN PLACE / VALIDÉ:
@@ -533,196 +544,196 @@
 - kill switch + DRP finalisés</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>évolutivité de l'infrastructure</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>L'infrastructure est évolutive : l'intégration d'autres sites est simple et rapide.</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>choix_infrastructure</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Les éléments de la pile technique choisie sont pris en charge par la communauté et régulièrement mis à jour.</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>livraison_diagramme</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Un schéma d'infrastructure est présenté lors de la première revue.</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>qualité_diagramme</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Le schéma d'infrastructure comprend les deux sites et leurs réseaux, les points de contrôle, le VPN, le bastion, le transfert DNS, les outils de gestion IP et l'observabilité.</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>iac_livraison</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>La plupart des ressources sont déployées à l'aide de l'infrastructure en tant que code.</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>qualité_iac</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Le code définissant l'infrastructure est lisible et respecte les meilleures pratiques.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="240" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>spécification_réseau1</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Le site sur site n'est accessible qu'en interne et les étudiants peuvent en faire la démonstration.</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>EXPLICATION: Site web interne (nginx sur bastion 192.168.10.11, LAN 192.168.10.0/24). Accessible uniquement depuis réseau interne/VPN, non exposé sur Internet.
 PREUVE COMPLÈTE (2026-05-28):
@@ -738,75 +749,75 @@
 6) Reconnecter VPN et refaire étape 2</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="11" ht="208" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>spécification_réseau2</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Le site distant est accessible de l'extérieur et les étudiants peuvent en faire la démonstration.</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>EXPLICATION: Le site distant doit être accessible depuis l'extérieur de façon contrôlée. Ici: accès via VPN puis bastion SSH (moindre privilège). Accès direct aux VMs internes depuis Internet non souhaité.
-PREUVE (2026-05-28):
-- site distant joignable via VPN
-- administration via bastion confirmée
-- NAT pfSense WAN:22 -&gt; 192.168.10.11:22 configuré
-- NAT routeur amont (78.202.114.212:22 -&gt; 192.168.102.103:22) en attente chez le pote pour démo 100% Internet sans VPN
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Accès externe au site distant via bastion SSH. Port 22 public bloqué; redirection box TCP 2222 -&gt; pfSense -&gt; bastion.
+PREUVE (2026-05-29):
+- nc -vz 78.202.114.212 2222 -&gt; succeeded
+- nc -vz 78.202.114.212 22 -&gt; timeout (normal, port non exposé)
+- ssh -p 2222 bastion@78.202.114.212 -&gt; handshake SSH OK (Permission denied sans mot de passe = service joignable)
 COMMANDES DÉMO:
-1) ssh bastion@192.168.102.103
-2) ping -c 3 192.168.10.10
-3) (après NAT box) ssh bastion@78.202.114.212</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
+1) nc -vz -G 5 78.202.114.212 2222
+2) ssh -p 2222 bastion@78.202.114.212
+3) (VPN) ssh bastion@192.168.102.103
+4) ping -c 3 192.168.10.10 depuis bastion</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="12" ht="224" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>réseau_vpn</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Les deux sites sont interconnectés via un VPN sécurisé.</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>EXPLICATION: Le VPN (OpenVPN) crée un tunnel chifré entre ton Mac et le site distant. Sans VPN tu n'accèdes pas aux IP privées (192.168.10.x). Avec VPN tu passes par le réseau tunnel (ex. 10.8.0.1).
 PREUVE (2026-05-28):
@@ -821,34 +832,34 @@
 4) traceroute 192.168.102.11</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="13" ht="304" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>pare-feu réseau</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Chaque site est équipé d'un pare-feu : ils sont correctement configurés, notamment pour la séparation du trafic. Les étudiants peuvent en démontrer l'efficacité.</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>EXPLICATION: pfSense (VM 100) filtre le trafic WAN/LAN. On démontre flux autorisé vs bloqué. Double NAT: box (78.202.114.212) -&gt; pfSense (192.168.102.103) -&gt; bastion (192.168.10.11).
 PREUVE PARTIELLE (2026-05-28):
@@ -864,37 +875,38 @@
 1) nc -vzu 78.202.114.212 1194
 2) nc -vz -G 3 78.202.114.212 80
 3) nc -vz -G 3 192.168.102.103 22
-4) (après NAT box) nc -vz -G 3 78.202.114.212 22</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+4) (après NAT box) nc -vz -G 3 78.202.114.212 22
+MAJ 2026-05-29: TCP/2222 public OK (bastion), TCP/22 public timeout, UDP/1194 OK.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="224" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>réseau_dns</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Une redirection DNS existe entre les deux sites.</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>EXPLICATION DNS:
 - DNS = annuaire nom -&gt; IP
@@ -910,88 +922,88 @@
 3) nslookup client1.site2.local 192.168.10.1</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>gestion_ip_réseau</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>La gestion des adresses IP est automatisée via un IPAM, qui est mis à jour automatiquement.</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>accès_sec</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Le principe du moindre privilège est correctement mis en œuvre.</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="192" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>sec_bastion</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>L'accès au site distant est sécurisé par la mise en place d'un bastion.</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>EXPLICATION: Le bastion (VM 102, 192.168.10.11) est un sas SSH: seule porte d'entrée admin depuis l'extérieur. On évite d'exposer directement les VMs internes (client 101). Chaîne: Internet -&gt; pfSense NAT TCP/22 -&gt; bastion -&gt; réseau interne.
 PREUVE (2026-05-28):
@@ -1004,363 +1016,363 @@
 4) (après NAT box) ssh bastion@78.202.114.212</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>identifiants sec</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>La gestion des identifiants et des secrets est correctement sécurisée (coffre-fort numérique, chiffrement, etc.).</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>incident_killswitch</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Il existe une stratégie d'arrêt d'urgence (interrupteur coupe-circuit) qui n'empêche pas la récupération.</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>incident_recovery</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>La stratégie de reprise après sinistre est utilisable et reproductible : elle spécifie les étapes à suivre pour reconstruire l'infrastructure.</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>centralisation des journaux</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Les journaux de tous les composants de l'infrastructure sont centralisés.</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>observabilité des journaux</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>L'observabilité complète (journaux + indicateurs + traces) permet une surveillance en temps réel de tous les composants de l'infrastructure.</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>analyse des journaux</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>L'analyse des données de télémétrie est pertinente.</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>journal_visuals</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>L'analyse des données de télémétrie est améliorée grâce aux représentations visuelles.</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>pratiques de dépôt</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Les étudiants utilisent un outil de gestion de versions avec un flux de travail approprié, comprenant une stratégie de branchement, des commits réguliers, des messages descriptifs et un fichier gitignore.</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>document_dépôt</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Le dépôt contient une documentation claire, structurée et compréhensible.</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>contenu du dépôt</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Le dépôt contient le code source et les configurations des composants (machines virtuelles, réseaux, outils).</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>proj_subdivision</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>La subdivision du projet en phases est représentée visuellement par un diagramme de Gantt ou équivalent, présenté lors de la première revue et mis à jour régulièrement.</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>planification_projet</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Lors de la première revue, un backlog comprenant les tâches à accomplir et leur répartition au sein de l'équipe est présenté et mis à jour régulièrement.</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>présentation_projet</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Le projet est présenté de manière professionnelle en utilisant des supports pertinents (diapositives et/ou démonstration).</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>KO</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Haute</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
@@ -1378,7 +1390,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
feat(cia): architecture S2, IaC Ansible et livrables docs
Documente le labo site distant (IPs, pfSense, bastion), ajoute rôles Ansible,
configs NetBox/Elastic, scénarios de démo et met à jour la grille d'évaluation.
</commit_message>
<xml_diff>
--- a/docs/criteres_evaluation_infrastructure.xlsx
+++ b/docs/criteres_evaluation_infrastructure.xlsx
@@ -525,23 +525,14 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>EXPLICATION: Services requis du sujet CIA: 2 sites Proxmox, VPN, 2x pfSense, bastion, DNS, IPAM NetBox, Elastic, site web interne.
-DÉJÀ EN PLACE / VALIDÉ:
-- Proxmox + VMs 100(FW) 101(Client) 102(Bastion)
-- OpenVPN site-to-site/client
-- pfSense + règles NAT
-- Bastion SSH
-- DNS forwarding + host override
-RESTE:
-- NetBox IPAM auto
-- centralisation logs Elastic
-- site web interne only
-- kill switch + DRP finalisés</t>
+          <t>EXPLICATION: Site S2 hybride opérationnel (VPN, pfSense, 3 VMs).
+PREUVE: architecture.md, critères réseau OK.
+MANQUE: site S1 services complets (NetBox, Elastic).</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -551,7 +542,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -568,7 +559,14 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Convention site N dans architecture.md.
+PREUVE: section Évolutivité.
+MANQUE: exemple 3e site fictif dans NetBox.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -578,7 +576,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -595,7 +593,14 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Stack Proxmox/pfSense/OpenVPN/NetBox/Elastic documentée README.
+PREUVE: README pile technique.
+MANQUE: tableau versions figées.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -605,7 +610,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -622,7 +627,14 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Schéma Mermaid versionné + export PNG à joindre.
+PREUVE: docs/architecture-diagram.mmd, docs/architecture.md.
+MANQUE: capture PNG/SVG exportée dans docs/ pour soutenance.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -632,7 +644,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -649,7 +661,14 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Diagramme décrit sites S1/S2, VPN, bastion, flux WAN.
+PREUVE: architecture.md section Mermaid.
+MANQUE: relecture encadrant + export image haute résolution.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -659,7 +678,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -676,7 +695,14 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Playbooks site.yml, netbox-sync.yml + rôles common/bastion/netbox_sync.
+PREUVE: iac/ansible/playbooks/, roles/.
+COMMANDES: ansible-playbook playbooks/site.yml --check</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -686,7 +712,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -703,7 +729,13 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Rôles modulaires, inventaire exemple, dry-run NetBox.
+MANQUE: exécution réelle sur production.yml + NetBox live.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -713,7 +745,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -946,7 +978,14 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Modèle YAML + script API NetBox + playbook sync.
+PREUVE: configs/netbox/sites-prefixes.example.yml, scripts/sync_from_inventory.py.
+MANQUE: instance NetBox S1 déployée + sync non dry-run.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -956,7 +995,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -973,7 +1012,14 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Matrice moindre privilège documentée.
+PREUVE: docs/secrets-and-access.md, bastion dédié, pas de root SSH public.
+MANQUE: coffre équipe formalisé en soutenance.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -983,7 +1029,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1086,14 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Secrets hors Git (.gitignore), tokens via env.
+PREUVE: .gitignore, secrets-and-access.md.
+MANQUE: démo coffre (sans afficher mdp).</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1050,7 +1103,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1120,14 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Procédure S2 dans drp-runbook (WAN UDP 1194).
+PREUVE: docs/drp-runbook.md section Site 2.
+MANQUE: test chronométré + captures.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1077,7 +1137,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1154,14 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Ordre reconstruction documenté.
+PREUVE: drp-runbook.md ordre 1-9.
+MANQUE: exercice DRP réel.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1104,7 +1171,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1296,14 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Conventions branches/commits, .gitignore secrets, historique main.
+PREUVE: docs/git-workflow.md, .gitignore (*.ovpn, production.yml).
+COMMANDES: git log --oneline -5</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1239,7 +1313,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1330,14 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>EXPLICATION: README principal + docs architecture, demo, DRP, secrets.
+PREUVE: README.md, docs/architecture.md, docs/demo-scenarios.md.
+COMMANDES: ouvrir README sur GitHub.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1266,7 +1347,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1364,14 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Dépôt structuré iac/, configs/, apps/, docs/, legacy/.
+PREUVE: arborescence README + playbooks Ansible + configs pfSense/NetBox/Elastic.
+COMMANDES: tree -L 2 ou parcours GitHub.</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1293,7 +1381,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1425,14 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Phases F0-F7 avec statuts dans gantt.md.
+PREUVE: docs/gantt.md journal décisions.
+MANQUE: lien GitHub Projects si exigé.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1347,7 +1442,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(cia): NetBox, Elastic, Filebeat, diagramme PNG et deploy labo
Ajoute stacks Docker S1, playbooks Ansible complets, script kill switch,
guide deploy-lab, architecture S1 et mise à jour grille d'évaluation.
</commit_message>
<xml_diff>
--- a/docs/criteres_evaluation_infrastructure.xlsx
+++ b/docs/criteres_evaluation_infrastructure.xlsx
@@ -493,12 +493,14 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>EXPLICATION: Infrastructure hybride = 2 sites Proxmox interconnectés VPN, sécurisés, observables. Partiellement fonctionnelle (VPN+bastion+DNS OK sur site distant). Manque site A complet, services transverses (NetBox/Elastic), démo bout-en-bout documentée.</t>
+          <t>EXPLICATION: Hybride S2 live ; S1 automatisé en attente VM svc-s1.
+PREUVE: deploy-lab.md checklist.
+MANQUE: démo live NetBox+Kibana.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -508,7 +510,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -530,9 +532,9 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>EXPLICATION: Site S2 hybride opérationnel (VPN, pfSense, 3 VMs).
-PREUVE: architecture.md, critères réseau OK.
-MANQUE: site S1 services complets (NetBox, Elastic).</t>
+          <t>EXPLICATION: S2 opérationnel ; S1 documenté avec NetBox/Elastic prêts à déployer.
+PREUVE: architecture.md sites S1+S2.
+MANQUE: exécution deploy-site1 sur VM svc-s1.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -559,14 +561,14 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>EN COURS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EXPLICATION: Convention site N dans architecture.md.
-PREUVE: section Évolutivité.
-MANQUE: exemple 3e site fictif dans NetBox.</t>
+          <t>EXPLICATION: Convention site N + préfixes NetBox multi-sites dans YAML.
+PREUVE: architecture.md section Évolutivité, sites-prefixes.example.yml.
+COMMANDES: montrer entrées site1/site2 NetBox.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -576,7 +578,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -593,14 +595,14 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>EN COURS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>EXPLICATION: Stack Proxmox/pfSense/OpenVPN/NetBox/Elastic documentée README.
-PREUVE: README pile technique.
-MANQUE: tableau versions figées.</t>
+          <t>EXPLICATION: Stack Proxmox, pfSense, OpenVPN, NetBox, Elastic, Ansible, Docker documentée.
+PREUVE: README pile technique + versions compose (NetBox v4.1, ES 8.13).
+COMMANDES: README.md.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -610,7 +612,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -627,14 +629,14 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>EN COURS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EXPLICATION: Schéma Mermaid versionné + export PNG à joindre.
-PREUVE: docs/architecture-diagram.mmd, docs/architecture.md.
-MANQUE: capture PNG/SVG exportée dans docs/ pour soutenance.</t>
+          <t>EXPLICATION: Schéma d'architecture livré en PNG pour la soutenance.
+PREUVE: docs/architecture-diagram.png (généré depuis .mmd).
+COMMANDES: ouvrir PNG + docs/architecture.md.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -644,7 +646,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -661,14 +663,14 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>EN COURS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EXPLICATION: Diagramme décrit sites S1/S2, VPN, bastion, flux WAN.
-PREUVE: architecture.md section Mermaid.
-MANQUE: relecture encadrant + export image haute résolution.</t>
+          <t>EXPLICATION: Diagramme hybride S1/S2, VPN, bastion, services centralisés.
+PREUVE: architecture-diagram.png, cohérent avec architecture.md.
+COMMANDES: comparaison oral + schéma.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -678,7 +680,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -695,14 +697,14 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>EN COURS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EXPLICATION: Playbooks site.yml, netbox-sync.yml + rôles common/bastion/netbox_sync.
-PREUVE: iac/ansible/playbooks/, roles/.
-COMMANDES: ansible-playbook playbooks/site.yml --check</t>
+          <t>EXPLICATION: Playbooks deploy-site1, deploy-observability, netbox-sync, rôles Docker/NetBox/Elastic/Filebeat.
+PREUVE: iac/ansible/playbooks/, iac/docker/.
+COMMANDES: ansible-playbook playbooks/deploy-site1.yml --check</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -712,7 +714,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -729,13 +731,14 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>EN COURS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EXPLICATION: Rôles modulaires, inventaire exemple, dry-run NetBox.
-MANQUE: exécution réelle sur production.yml + NetBox live.</t>
+          <t>EXPLICATION: Rôles modulaires, variables vault, compose versionnés, inventaire exemple IPs réelles.
+PREUVE: group_vars/, roles/docker_host, netbox_stack, elastic_stack, filebeat.
+COMMANDES: voir docs/deploy-lab.md.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -745,7 +748,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -978,14 +981,14 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>EN COURS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EXPLICATION: Modèle YAML + script API NetBox + playbook sync.
-PREUVE: configs/netbox/sites-prefixes.example.yml, scripts/sync_from_inventory.py.
-MANQUE: instance NetBox S1 déployée + sync non dry-run.</t>
+          <t>EXPLICATION: NetBox Docker S1 + modèle YAML sites/préfixes/IP + script sync API + playbook.
+PREUVE: iac/docker/netbox/, configs/netbox/scripts/sync_from_inventory.py.
+COMMANDES: deploy-site1 puis NETBOX_URL/TOKEN + sync script.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -995,7 +998,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -1012,14 +1015,14 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>EN COURS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EXPLICATION: Matrice moindre privilège documentée.
-PREUVE: docs/secrets-and-access.md, bastion dédié, pas de root SSH public.
-MANQUE: coffre équipe formalisé en soutenance.</t>
+          <t>EXPLICATION: Matrice moindre privilège, bastion dédié, secrets hors Git.
+PREUVE: docs/secrets-and-access.md.
+COMMANDES: .gitignore + oral.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1029,7 +1032,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -1086,14 +1089,14 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>EN COURS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>EXPLICATION: Secrets hors Git (.gitignore), tokens via env.
-PREUVE: .gitignore, secrets-and-access.md.
-MANQUE: démo coffre (sans afficher mdp).</t>
+          <t>EXPLICATION: vault.yml / env vars, tokens NetBox API, pas de mdp dans Git.
+PREUVE: group_vars vault_*, deploy-lab.md.
+COMMANDES: montrer coffre équipe.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1103,7 +1106,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -1125,9 +1128,9 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>EXPLICATION: Procédure S2 dans drp-runbook (WAN UDP 1194).
-PREUVE: docs/drp-runbook.md section Site 2.
-MANQUE: test chronométré + captures.</t>
+          <t>EXPLICATION: Script scripts/kill-switch-s2.sh + procédure pfSense WAN UDP 1194 dans drp-runbook.
+PREUVE: drp-runbook.md, deploy-lab.md §3.
+MANQUE: test chronométré &lt;10min + captures (labo VPN actif).</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1154,14 +1157,14 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>EN COURS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>EXPLICATION: Ordre reconstruction documenté.
-PREUVE: drp-runbook.md ordre 1-9.
-MANQUE: exercice DRP réel.</t>
+          <t>EXPLICATION: Ordre reconstruction 1-9 + stacks Docker reproductibles.
+PREUVE: drp-runbook.md, deploy-site1.yml.
+COMMANDES: relire runbook oral.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1171,7 +1174,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1191,14 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Elasticsearch S1 + Filebeat bastion S2 (auth.log, nginx).
+PREUVE: rôle filebeat, elastic compose, deploy-observability.yml.
+COMMANDES: deploy-observability.yml puis logger test sur bastion.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1198,7 +1208,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1225,14 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Kibana sur svc-s1:5601, guide Discover/dashboards.
+PREUVE: configs/elastic/kibana-guide.md.
+COMMANDES: Kibana Discover filtre site:site2.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1225,7 +1242,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1259,14 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Procédure analyse SSH/nginx dans kibana-guide (filtres, histogrammes).
+PREUVE: kibana-guide.md section Discover.
+COMMANDES: recherche CIA-KIBANA-TEST après logger.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1252,7 +1276,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1293,14 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>EN COURS</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>EXPLICATION: Dashboard Kibana documenté ; export saved objects à joindre au rapport.
+PREUVE: kibana-guide.md.
+MANQUE: capture écran dashboard après déploiement Elastic.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1279,7 +1310,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Partiel</t>
         </is>
       </c>
     </row>
@@ -1301,9 +1332,9 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>EXPLICATION: Conventions branches/commits, .gitignore secrets, historique main.
-PREUVE: docs/git-workflow.md, .gitignore (*.ovpn, production.yml).
-COMMANDES: git log --oneline -5</t>
+          <t>EXPLICATION: git-workflow, commits conventionnels, secrets ignorés.
+PREUVE: docs/git-workflow.md, historique main.
+COMMANDES: git log --oneline.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1335,9 +1366,9 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>EXPLICATION: README principal + docs architecture, demo, DRP, secrets.
-PREUVE: README.md, docs/architecture.md, docs/demo-scenarios.md.
-COMMANDES: ouvrir README sur GitHub.</t>
+          <t>EXPLICATION: README, architecture, deploy-lab, demo-scenarios, DRP.
+PREUVE: docs/.
+COMMANDES: README + deploy-lab.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1369,9 +1400,9 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>EXPLICATION: Dépôt structuré iac/, configs/, apps/, docs/, legacy/.
-PREUVE: arborescence README + playbooks Ansible + configs pfSense/NetBox/Elastic.
-COMMANDES: tree -L 2 ou parcours GitHub.</t>
+          <t>EXPLICATION: iac/docker, scripts, configs, docs, apps complets.
+PREUVE: arborescence README.
+COMMANDES: parcours GitHub.</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1425,14 +1456,14 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>EN COURS</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>EXPLICATION: Phases F0-F7 avec statuts dans gantt.md.
-PREUVE: docs/gantt.md journal décisions.
-MANQUE: lien GitHub Projects si exigé.</t>
+          <t>EXPLICATION: Gantt F0-F7 à jour avec jalons et backlog labo.
+PREUVE: docs/gantt.md.
+COMMANDES: présenter phases soutenance.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1442,7 +1473,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>Oui</t>
         </is>
       </c>
     </row>

</xml_diff>